<commit_message>
Excel: colonna Blocco (schermata) nella checklist, budget Base via Zara 10/25
</commit_message>
<xml_diff>
--- a/catalogo/catalogo-governante.xlsx
+++ b/catalogo/catalogo-governante.xlsx
@@ -11642,7 +11642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -11650,6 +11650,7 @@
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -11678,6 +11679,11 @@
           <t>Minuti circa</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Blocco (schermata)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -11701,6 +11707,11 @@
       <c r="E2" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>Letto e biancheria</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -11724,6 +11735,11 @@
       <c r="E3" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>Letto e biancheria</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -11747,6 +11763,11 @@
       <c r="E4" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -11770,6 +11791,11 @@
       <c r="E5" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -11793,6 +11819,11 @@
       <c r="E6" s="2" t="n">
         <v>4</v>
       </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -11816,6 +11847,11 @@
       <c r="E7" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -11839,6 +11875,11 @@
       <c r="E8" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -11862,6 +11903,11 @@
       <c r="E9" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -11885,6 +11931,11 @@
       <c r="E10" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -11908,6 +11959,11 @@
       <c r="E11" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -11931,6 +11987,11 @@
       <c r="E12" s="2" t="n">
         <v>6</v>
       </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Pavimenti e controllo finale</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -11954,6 +12015,11 @@
       <c r="E13" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>Pavimenti e controllo finale</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -11977,6 +12043,11 @@
       <c r="E14" s="4" t="n">
         <v>8</v>
       </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Letto e biancheria</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -12000,6 +12071,11 @@
       <c r="E15" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>Letto e biancheria</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -12023,6 +12099,11 @@
       <c r="E16" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Letto e biancheria</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -12046,6 +12127,11 @@
       <c r="E17" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>Letto e biancheria</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -12069,6 +12155,11 @@
       <c r="E18" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -12092,6 +12183,11 @@
       <c r="E19" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -12115,6 +12211,11 @@
       <c r="E20" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -12138,6 +12239,11 @@
       <c r="E21" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -12161,6 +12267,11 @@
       <c r="E22" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -12184,6 +12295,11 @@
       <c r="E23" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -12207,6 +12323,11 @@
       <c r="E24" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>Pavimenti e controllo finale</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -12230,6 +12351,11 @@
       <c r="E25" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Alla partenza</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -12253,6 +12379,11 @@
       <c r="E26" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -12276,6 +12407,11 @@
       <c r="E27" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -12299,6 +12435,11 @@
       <c r="E28" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -12322,6 +12463,11 @@
       <c r="E29" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -12345,6 +12491,11 @@
       <c r="E30" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -12368,6 +12519,11 @@
       <c r="E31" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -12391,6 +12547,11 @@
       <c r="E32" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -12414,6 +12575,11 @@
       <c r="E33" s="6" t="n">
         <v>10</v>
       </c>
+      <c r="F33" s="18" t="inlineStr">
+        <is>
+          <t>Alla partenza</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -12437,6 +12603,11 @@
       <c r="E34" s="10" t="n">
         <v>12</v>
       </c>
+      <c r="F34" s="18" t="inlineStr">
+        <is>
+          <t>Pavimenti e controllo finale</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -12460,6 +12631,11 @@
       <c r="E35" s="10" t="n">
         <v>8</v>
       </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -12483,6 +12659,11 @@
       <c r="E36" s="10" t="n">
         <v>6</v>
       </c>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -12506,6 +12687,11 @@
       <c r="E37" s="10" t="n">
         <v>4</v>
       </c>
+      <c r="F37" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -12529,6 +12715,11 @@
       <c r="E38" s="10" t="n">
         <v>10</v>
       </c>
+      <c r="F38" s="18" t="inlineStr">
+        <is>
+          <t>Letto e biancheria</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -12552,6 +12743,11 @@
       <c r="E39" s="10" t="n">
         <v>6</v>
       </c>
+      <c r="F39" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -12575,6 +12771,11 @@
       <c r="E40" s="10" t="n">
         <v>6</v>
       </c>
+      <c r="F40" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -12598,6 +12799,7 @@
       <c r="E41" s="10" t="n">
         <v>10</v>
       </c>
+      <c r="F41" s="18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12708,7 +12910,7 @@
       </c>
       <c r="E3" s="18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+10 (igiene, una o due cose)</t>
         </is>
       </c>
       <c r="F3" s="18" t="inlineStr">
@@ -12740,7 +12942,7 @@
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+10 (igiene, una o due cose)</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
@@ -12860,7 +13062,7 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>+10 (una cosa di igiene)</t>
+          <t>+25 (igiene, prima dalla riga 'una per volta')</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
@@ -12892,7 +13094,7 @@
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>+10 (una cosa di igiene)</t>
+          <t>+25 (igiene, prima dalla riga 'una per volta')</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
@@ -13282,7 +13484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13449,6 +13651,18 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Blocco (schermata)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Nel foglio Checklist signora: il titolo grande sotto cui la riga compare sul telefono della signora (Letto e biancheria · Bagno · Camera · Cucina · Alla partenza · Pavimenti e controllo finale). Ogni blocco ha un solo tasto Fatto; le stelle si toccano una per una.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Catalogo: calendario vero a due signore (risposte di Michele), M08 chiusura estiva, M07 su tutte le camere
</commit_message>
<xml_diff>
--- a/catalogo/catalogo-governante.xlsx
+++ b/catalogo/catalogo-governante.xlsx
@@ -12812,7 +12812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12863,27 +12863,27 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Via Trento 47</t>
+          <t>Via Zara 1° piano</t>
         </is>
       </c>
       <c r="C2" s="18" t="inlineStr">
         <is>
-          <t>Ripasso</t>
+          <t>Ripasso base (leggerissimo)</t>
         </is>
       </c>
       <c r="D2" s="18" t="inlineStr">
         <is>
-          <t>Signora Appartamenti</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E2" s="18" t="inlineStr">
         <is>
-          <t>+15</t>
+          <t>+10 (igiene, una o due cose)</t>
         </is>
       </c>
       <c r="F2" s="18" t="inlineStr">
         <is>
-          <t>Profilo Lusso</t>
+          <t>Profilo Base (operai)</t>
         </is>
       </c>
     </row>
@@ -12895,17 +12895,17 @@
       </c>
       <c r="B3" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 1° piano</t>
+          <t>Via Zara 2° piano</t>
         </is>
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>Ripasso base</t>
+          <t>Ripasso base (leggerissimo)</t>
         </is>
       </c>
       <c r="D3" s="18" t="inlineStr">
         <is>
-          <t>Signora Appartamenti</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E3" s="18" t="inlineStr">
@@ -12927,27 +12927,27 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 2° piano</t>
+          <t>Via Trento 47</t>
         </is>
       </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
-          <t>Ripasso base</t>
+          <t>Ripasso (più impegnativo, ma sempre ripasso)</t>
         </is>
       </c>
       <c r="D4" s="18" t="inlineStr">
         <is>
-          <t>Signora Appartamenti</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>+10 (igiene, una o due cose)</t>
+          <t>+15</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Profilo Base (operai)</t>
+          <t>Profilo Lusso</t>
         </is>
       </c>
     </row>
@@ -12977,7 +12977,11 @@
           <t>+15 a camera</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr"/>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Solo le camere occupate (es. Fenicotteri salta se Salerno non c'è)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
@@ -12997,7 +13001,7 @@
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Signora 2° piano [CONTROLLA: è lei o la signora del 1° piano?]</t>
+          <t>Signora 2° piano</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -13025,7 +13029,7 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Signora Appartamenti</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
@@ -13057,7 +13061,7 @@
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Signora Appartamenti</t>
+          <t>Signora 1° piano (insieme alla signora del 2° piano)</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
@@ -13067,7 +13071,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Profilo Base</t>
+          <t>Profilo Base · le due signore lavorano insieme</t>
         </is>
       </c>
     </row>
@@ -13089,7 +13093,7 @@
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Signora Appartamenti</t>
+          <t>Signora 1° piano (insieme alla signora del 2° piano)</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
@@ -13099,7 +13103,7 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Profilo Base</t>
+          <t>Profilo Base · le due signore lavorano insieme</t>
         </is>
       </c>
     </row>
@@ -13131,7 +13135,7 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>[CONTROLLA: venerdì o sabato?]</t>
+          <t>I tecnici vanno a casa il venerdì</t>
         </is>
       </c>
     </row>
@@ -13143,7 +13147,7 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Alba, Tramonto, Passerella, Fenicotteri</t>
+          <t>Alba, Tramonto, Fenicotteri</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
@@ -13161,11 +13165,7 @@
           <t>+30 a camera</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>[CONTROLLA: venerdì o sabato?]</t>
-        </is>
-      </c>
+      <c r="F11" s="18" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -13175,7 +13175,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Via Zara piano terra</t>
+          <t>Passerella, Lella</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -13185,17 +13185,17 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Signora Appartamenti</t>
+          <t>Signora 2° piano</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>+30</t>
+          <t>+30 a camera</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>[DECIDI: profilo Lusso o Base?]</t>
+          <t>Più scalinata, ingresso e zone comuni</t>
         </is>
       </c>
     </row>
@@ -13207,7 +13207,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Lella oppure Nicole</t>
+          <t>Nicole</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -13217,7 +13217,7 @@
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>[CONTROLLA chi]</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
@@ -13225,11 +13225,7 @@
           <t>+30</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>Tutte e due devono restare ben pulite: Nicole quando?</t>
-        </is>
-      </c>
+      <c r="F13" s="18" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
@@ -13239,7 +13235,7 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Il resto delle totali ('ognuna ha le sue cose')</t>
+          <t>Via Zara piano terra</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -13249,15 +13245,19 @@
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>[COMPLETA]</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>+30 a camera</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr"/>
+          <t>+30</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>[DECIDI: profilo Lusso o Base?]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
@@ -13288,6 +13288,13 @@
       <c r="F15" s="18" t="inlineStr">
         <is>
           <t>Mai di domenica</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Da ottobre a maggio (inverno): questi giorni fissi, con due signore (la signora del 1° piano fa anche gli appartamenti). Da giugno ad agosto (estate): niente giorni fissi, le pulizie seguono arrivi e partenze del prospetto; le stelle vanno sulle pulizie di partenza, 1-2 a partenza, prima il visibile. Due finestre di reset: fine maggio (M07) e inizio settembre (M08).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catalogo: calendario vero, giovedì via Zara 2° alla signora del 2° piano (una per appartamento, 10 €)
</commit_message>
<xml_diff>
--- a/catalogo/catalogo-governante.xlsx
+++ b/catalogo/catalogo-governante.xlsx
@@ -12883,7 +12883,7 @@
       </c>
       <c r="F2" s="18" t="inlineStr">
         <is>
-          <t>Profilo Base (operai)</t>
+          <t>Modo Operai</t>
         </is>
       </c>
     </row>
@@ -12915,7 +12915,7 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Profilo Base (operai)</t>
+          <t>Modo Operai</t>
         </is>
       </c>
     </row>
@@ -12947,7 +12947,7 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Profilo Lusso</t>
+          <t>Modo Tecnici</t>
         </is>
       </c>
     </row>
@@ -13039,7 +13039,7 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Profilo Lusso</t>
+          <t>Modo Tecnici</t>
         </is>
       </c>
     </row>
@@ -13061,7 +13061,7 @@
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano (insieme alla signora del 2° piano)</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
@@ -13071,7 +13071,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Profilo Base · le due signore lavorano insieme</t>
+          <t>Modo Operai · le due signore lavorano insieme</t>
         </is>
       </c>
     </row>
@@ -13093,7 +13093,7 @@
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano (insieme alla signora del 2° piano)</t>
+          <t>Signora 2° piano</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
@@ -13103,7 +13103,7 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Profilo Base · le due signore lavorano insieme</t>
+          <t>Modo Operai · le due signore lavorano insieme</t>
         </is>
       </c>
     </row>
@@ -13291,6 +13291,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Catalogo 0.34: via Zara 1° e 2° piano unito, giovedì in due (sotto/sopra), blocco Piano di sopra
</commit_message>
<xml_diff>
--- a/catalogo/catalogo-governante.xlsx
+++ b/catalogo/catalogo-governante.xlsx
@@ -11642,7 +11642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12582,30 +12582,26 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>BASE · ripasso (via Zara 1° e 2°, operai)</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>Pavimenti scopati e lavati (camere, bagno, cucina)</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>C52, B34, K13</t>
-        </is>
-      </c>
-      <c r="E34" s="10" t="n">
-        <v>12</v>
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>APPARTAMENTO · aggiunte cucina</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Piano di sopra (solo via Zara 1° e 2°): camere e bagno di sopra come quelli di sotto</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr"/>
+      <c r="E34" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="F34" s="18" t="inlineStr">
         <is>
-          <t>Pavimenti e controllo finale</t>
+          <t>Piano di sopra</t>
         </is>
       </c>
     </row>
@@ -12616,24 +12612,24 @@
         </is>
       </c>
       <c r="B35" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Bagno: WC, lavandino, doccia con capelli via dalla piletta</t>
+          <t>Pavimenti scopati e lavati (camere, bagno, cucina)</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>B17, B12, B23</t>
+          <t>C52, B34, K13</t>
         </is>
       </c>
       <c r="E35" s="10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F35" s="18" t="inlineStr">
         <is>
-          <t>Bagno</t>
+          <t>Pavimenti e controllo finale</t>
         </is>
       </c>
     </row>
@@ -12644,24 +12640,24 @@
         </is>
       </c>
       <c r="B36" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Cucina: piano, fornelli, lavello (i piatti sporchi degli ospiti no)</t>
+          <t>Bagno: WC, lavandino, doccia con capelli via dalla piletta</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>K05, K03, K06</t>
+          <t>B17, B12, B23</t>
         </is>
       </c>
       <c r="E36" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>Cucina</t>
+          <t>Bagno</t>
         </is>
       </c>
     </row>
@@ -12672,20 +12668,20 @@
         </is>
       </c>
       <c r="B37" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Bidoni: svuotati, sciacquati, fuori secondo il calendario; cestini</t>
+          <t>Cucina: piano, fornelli, lavello (i piatti sporchi degli ospiti no)</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>K12, C51, B32</t>
+          <t>K05, K03, K06</t>
         </is>
       </c>
       <c r="E37" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
@@ -12696,56 +12692,56 @@
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>BASE · totale (giovedì)</t>
+          <t>BASE · ripasso (via Zara 1° e 2°, operai)</t>
         </is>
       </c>
       <c r="B38" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Come il ripasso + letti cambiati, asciugamani, coprimaterasso se macchiato</t>
+          <t>Bidoni: svuotati, sciacquati, fuori secondo il calendario; cestini</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>C31, B33, C30</t>
+          <t>K12, C51, B32</t>
         </is>
       </c>
       <c r="E38" s="10" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F38" s="18" t="inlineStr">
         <is>
-          <t>Letto e biancheria</t>
+          <t>Cucina</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>BASE · totale (giovedì)</t>
+          <t>BASE · ripasso (via Zara 1° e 2°, operai)</t>
         </is>
       </c>
       <c r="B39" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Bagno completo con antimuffa sul silicone e acqua bollente negli scarichi</t>
+          <t>Piano di sopra: letti rifatti, camere in ordine, bagno di sopra (WC, lavandino, doccia)</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>B08, B36, B18</t>
+          <t>C31, B17, B12, B23</t>
         </is>
       </c>
       <c r="E39" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F39" s="18" t="inlineStr">
         <is>
-          <t>Bagno</t>
+          <t>Piano di sopra</t>
         </is>
       </c>
     </row>
@@ -12756,24 +12752,24 @@
         </is>
       </c>
       <c r="B40" s="10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Cucina: microonde, frigo guardato, piastrelle dietro i fornelli</t>
+          <t>Come il ripasso + letti cambiati, asciugamani, coprimaterasso se macchiato</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>K09, K08, K14</t>
+          <t>C31, B33, C30</t>
         </is>
       </c>
       <c r="E40" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F40" s="18" t="inlineStr">
         <is>
-          <t>Cucina</t>
+          <t>Letto e biancheria</t>
         </is>
       </c>
     </row>
@@ -12784,22 +12780,106 @@
         </is>
       </c>
       <c r="B41" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>Bagno completo con antimuffa sul silicone e acqua bollente negli scarichi</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>B08, B36, B18</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F41" s="18" t="inlineStr">
+        <is>
+          <t>Bagno</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>BASE · totale (giovedì)</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Cucina: microonde, frigo guardato, piastrelle dietro i fornelli</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>K09, K08, K14</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F42" s="18" t="inlineStr">
+        <is>
+          <t>Cucina</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>BASE · totale (giovedì)</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="C41" s="10" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
         <is>
           <t>Una cosa di igiene a rotazione (una per volta): filtri cappa, filtri condizionatore, forno, guarnizioni frigo, muffa negli angoli, scarichi</t>
         </is>
       </c>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="D43" s="10" t="inlineStr">
         <is>
           <t>K02, C03, K04, K08, B01, B35</t>
         </is>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E43" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="F41" s="18" t="inlineStr"/>
+      <c r="F43" s="18" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>BASE · totale (giovedì)</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Piano di sopra: letti cambiati, camere spolverate e pavimenti, bagno di sopra completo</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>C31, B33, C52, B34, B17, B12, B23</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F44" s="18" t="inlineStr">
+        <is>
+          <t>Piano di sopra</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12812,7 +12892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12863,7 +12943,7 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 1° piano</t>
+          <t>Via Zara 1° e 2° piano</t>
         </is>
       </c>
       <c r="C2" s="18" t="inlineStr">
@@ -12883,7 +12963,7 @@
       </c>
       <c r="F2" s="18" t="inlineStr">
         <is>
-          <t>Modo Operai</t>
+          <t>Modo Operai · un appartamento solo su due piani</t>
         </is>
       </c>
     </row>
@@ -12895,12 +12975,12 @@
       </c>
       <c r="B3" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 2° piano</t>
+          <t>Via Trento 47</t>
         </is>
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>Ripasso base (leggerissimo)</t>
+          <t>Ripasso (più impegnativo, ma sempre ripasso)</t>
         </is>
       </c>
       <c r="D3" s="18" t="inlineStr">
@@ -12910,44 +12990,44 @@
       </c>
       <c r="E3" s="18" t="inlineStr">
         <is>
-          <t>+10 (igiene, una o due cose)</t>
+          <t>+15</t>
         </is>
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Modo Operai</t>
+          <t>Modo Tecnici</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>Lunedì</t>
+          <t>Mercoledì</t>
         </is>
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>Via Trento 47</t>
+          <t>Alba, Tramonto, Passerella, Fenicotteri</t>
         </is>
       </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
-          <t>Ripasso (più impegnativo, ma sempre ripasso)</t>
+          <t>Ripasso</t>
         </is>
       </c>
       <c r="D4" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano</t>
+          <t>Signora 2° piano</t>
         </is>
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>+15</t>
+          <t>+15 a camera</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Modo Tecnici</t>
+          <t>Solo le camere occupate (es. Fenicotteri salta se Salerno non c'è)</t>
         </is>
       </c>
     </row>
@@ -12959,7 +13039,7 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Alba, Tramonto, Passerella, Fenicotteri</t>
+          <t>Lella</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
@@ -12974,42 +13054,42 @@
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>+15 a camera</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Solo le camere occupate (es. Fenicotteri salta se Salerno non c'è)</t>
-        </is>
-      </c>
+          <t>+15</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Mercoledì</t>
+          <t>Giovedì</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Lella</t>
+          <t>Via Trento 47</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Ripasso</t>
+          <t>Cambio totale (2 letti, 1 h – 1 h 15)</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Signora 2° piano</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>+15</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr"/>
+          <t>+30</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Modo Tecnici</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
@@ -13019,27 +13099,27 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Via Trento 47</t>
+          <t>Via Zara 1° e 2° piano · piano di sotto</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Cambio totale (2 letti, 1 h – 1 h 15)</t>
+          <t>Cambio totale base</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano</t>
+          <t>Signora 1° piano, insieme alla signora del 2° piano</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>+30</t>
+          <t>+25 (igiene, prima dalla riga 'una per volta')</t>
         </is>
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Modo Tecnici</t>
+          <t>Modo Operai · le due signore lavorano insieme, una per piano: 10 € a testa. Le stelle stanno sul piano di sotto</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13131,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 1° piano</t>
+          <t>Via Zara 1° e 2° piano · piano di sopra</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
@@ -13061,49 +13141,49 @@
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano</t>
+          <t>Signora 2° piano, insieme alla signora del 1° piano</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>+25 (igiene, prima dalla riga 'una per volta')</t>
+          <t>+0 (le stelle stanno sul piano di sotto)</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Modo Operai · le due signore lavorano insieme</t>
+          <t>Modo Operai · camere e bagno di sopra, 10 €</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>Giovedì</t>
+          <t>Venerdì</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 2° piano</t>
+          <t>Salvatore, Aurora, Michele, Antonio</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>Cambio totale base</t>
+          <t>Cambio totale, camera libera fino a lunedì</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Signora 2° piano</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>+25 (igiene, prima dalla riga 'una per volta')</t>
+          <t>+45 a camera (camera vuota: anche le cose 'a camera libera')</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Modo Operai · le due signore lavorano insieme</t>
+          <t>I tecnici vanno a casa il venerdì</t>
         </is>
       </c>
     </row>
@@ -13115,39 +13195,35 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Salvatore, Aurora, Michele, Antonio</t>
+          <t>Alba, Tramonto, Fenicotteri</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>Cambio totale, camera libera fino a lunedì</t>
+          <t>Cambio totale</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano</t>
+          <t>Signora 2° piano</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>+45 a camera (camera vuota: anche le cose 'a camera libera')</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>I tecnici vanno a casa il venerdì</t>
-        </is>
-      </c>
+          <t>+30 a camera</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>Venerdì</t>
+          <t>Sabato</t>
         </is>
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Alba, Tramonto, Fenicotteri</t>
+          <t>Passerella, Lella</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
@@ -13165,7 +13241,11 @@
           <t>+30 a camera</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr"/>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>Più scalinata, ingresso e zone comuni</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -13175,7 +13255,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Passerella, Lella</t>
+          <t>Nicole</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -13185,19 +13265,15 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Signora 2° piano</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>+30 a camera</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>Più scalinata, ingresso e zone comuni</t>
-        </is>
-      </c>
+          <t>+30</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
@@ -13207,7 +13283,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Nicole</t>
+          <t>Via Zara piano terra</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -13225,75 +13301,47 @@
           <t>+30</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr"/>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>[DECIDI: profilo Lusso o Base?]</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>Sabato</t>
+          <t>Domenica</t>
         </is>
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Via Zara piano terra</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>Cambio totale</t>
+          <t>Nessuna pulizia</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>+30</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>[DECIDI: profilo Lusso o Base?]</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Domenica</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>Nessuna pulizia</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
           <t>Mai di domenica</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Da ottobre a maggio (inverno): questi giorni fissi, con due signore (la signora del 1° piano fa anche gli appartamenti). Da giugno ad agosto (estate): niente giorni fissi, le pulizie seguono arrivi e partenze del prospetto; le stelle vanno sulle pulizie di partenza, 1-2 a partenza, prima il visibile. Due finestre di reset: fine maggio (M07) e inizio settembre (M08).</t>
         </is>

</xml_diff>

<commit_message>
Catalogo 0.35: giovedì via Zara a Lucia sola; specifiche punto 14 costruito, con le assunzioni da confermare
</commit_message>
<xml_diff>
--- a/catalogo/catalogo-governante.xlsx
+++ b/catalogo/catalogo-governante.xlsx
@@ -12892,7 +12892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 1° e 2° piano · piano di sotto</t>
+          <t>Via Zara 1° e 2° piano</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano, insieme alla signora del 2° piano</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
@@ -13119,39 +13119,39 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Modo Operai · le due signore lavorano insieme, una per piano: 10 € a testa. Le stelle stanno sul piano di sotto</t>
+          <t>Modo Operai · lo fa Lucia da sola, tutti e due i piani: 2 ore standard, 20 € (specifiche §14; Selena negli appartamenti non va mai)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>Giovedì</t>
+          <t>Venerdì</t>
         </is>
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Via Zara 1° e 2° piano · piano di sopra</t>
+          <t>Salvatore, Aurora, Michele, Antonio</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Cambio totale base</t>
+          <t>Cambio totale, camera libera fino a lunedì</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Signora 2° piano, insieme alla signora del 1° piano</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>+0 (le stelle stanno sul piano di sotto)</t>
+          <t>+45 a camera (camera vuota: anche le cose 'a camera libera')</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Modo Operai · camere e bagno di sopra, 10 €</t>
+          <t>I tecnici vanno a casa il venerdì</t>
         </is>
       </c>
     </row>
@@ -13163,39 +13163,35 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Salvatore, Aurora, Michele, Antonio</t>
+          <t>Alba, Tramonto, Fenicotteri</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>Cambio totale, camera libera fino a lunedì</t>
+          <t>Cambio totale</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano</t>
+          <t>Signora 2° piano</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>+45 a camera (camera vuota: anche le cose 'a camera libera')</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>I tecnici vanno a casa il venerdì</t>
-        </is>
-      </c>
+          <t>+30 a camera</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>Venerdì</t>
+          <t>Sabato</t>
         </is>
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Alba, Tramonto, Fenicotteri</t>
+          <t>Passerella, Lella</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -13213,7 +13209,11 @@
           <t>+30 a camera</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr"/>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>Più scalinata, ingresso e zone comuni</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -13223,7 +13223,7 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Passerella, Lella</t>
+          <t>Nicole</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
@@ -13233,19 +13233,15 @@
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>Signora 2° piano</t>
+          <t>Signora 1° piano</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>+30 a camera</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>Più scalinata, ingresso e zone comuni</t>
-        </is>
-      </c>
+          <t>+30</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -13255,7 +13251,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Nicole</t>
+          <t>Via Zara piano terra</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -13273,74 +13269,47 @@
           <t>+30</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr"/>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>[DECIDI: profilo Lusso o Base?]</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Sabato</t>
+          <t>Domenica</t>
         </is>
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Via Zara piano terra</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Cambio totale</t>
+          <t>Nessuna pulizia</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Signora 1° piano</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>+30</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>[DECIDI: profilo Lusso o Base?]</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Domenica</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>Nessuna pulizia</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
           <t>Mai di domenica</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Da ottobre a maggio (inverno): questi giorni fissi, con due signore (la signora del 1° piano fa anche gli appartamenti). Da giugno ad agosto (estate): niente giorni fissi, le pulizie seguono arrivi e partenze del prospetto; le stelle vanno sulle pulizie di partenza, 1-2 a partenza, prima il visibile. Due finestre di reset: fine maggio (M07) e inizio settembre (M08).</t>
         </is>

</xml_diff>